<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.001-01 La fraise de Chouchou
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.001-01.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.001-01.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jardin</t>
+          <t>jardin, treille, terre, soleil, fraise, fil de fer, bois, feuille de vigne, jus, ombre</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Chouchou trouve une fraise rouge. Il est content. Il nomme sa joie et partage un bout avec papa.</t>
+          <t>La treille du fond fait de l'ombre. Sur le bois, un éclat de treille luit. Chouchou veut la fraise, maintenant. Il attrape la feuille. Puis la fraise tiède. Sourire qui arrive. Poitrine pleine. Papa s'accroupit. Il dit je suis content. Un bout pour papa. Merci vécu. Deuxième ruse : fraise trop chaude, elle glisse. Il refuse de foncer. Un bout pour maman. Un éclat de treille tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un petit panier attend près du gravier. Dedans, un torchon à carreaux. Les fraisiers cachent des fruits. Les feuilles sont vertes. Un peu piquantes. La terre est chaude. L'arrosoir de papa goutte encore. Je pose le panier, Chouchou. On marche tout doux, entre les plants. Ça sent le sucre, papa. Oui. Les fraises sont mûres. Le soleil est doux, ce matin. Regarde sous les feuilles. En ce moment, Chouchou marche. Il est près des fraisiers. Papa est là, près de lui. Chouchou voit une fraise rouge. Une fraise ! Elle brille. Tu la cueilles tout doucement ? Une seule, pour commencer. Chouchou cueille la fraise. Tout doucement. La fraise sent le sucre. Elle est tiède dans sa main. Chouchou sent ses joues chaudes. Son ventre est léger. Un sourire arrive. Je suis content. C'est de la joie. Tu es content. Tes joues sont chaudes. Oui. De la joie. On peut partager. Chouchou tend la fraise. Un bout pour papa. Et un tout petit bout pour toi. Papa prend un tout petit bout. Chouchou prend un tout petit bout. Merci, Chouchou. Tu as partagé. Je suis content. La joie est là, dans le jardin. Ils sourient ensemble. La terre reste chaude. L'arrosoir goutte encore.</t>
+          <t>La treille du fond fait de l'ombre. Elle fait de l'ombre, papa. Tu la vois, la treille ? Oui, papa. Un fil de fer vibre sous le pouce. Ting, près du bois. Tu entends le fil, Chouchou ? Oui, maman. Maman s'assoit près du fil. La terre chauffe les genoux. Elle est chaude. Les genoux sont bien ? Oui, maman. Papa soulève une feuille de vigne. Le bois sent le soleil. Tu sens le bois chaud ? Oui, papa. Sur le bois, un éclat de treille luit. Il brille, maman. Tu le vois, sur le bois ? Oui, un petit point. Le soleil le touche. Un rayon glisse sur le bord. La treille chauffe le jardin. Elle est chaude. Tu poses la main, Chouchou ? Oui. Une fraise rouge attend sous la feuille. Une fraise ! Elle est rouge, Chouchou ? Oui, maman. Elle sent un peu le sucre. Ça sent le sucre, papa. Tu la veux, la fraise ? Oui, maintenant ! En ce moment, Chouchou tend la main. Je la prends, tout de suite ! Tout de suite ? Oui, papa. Chouchou attrape trop vite. Sa main prend la feuille. Oh. La fraise reste cachée. Les doigts tiennent du vert. La feuille, pas la fraise ? Pas la fraise. Chouchou reste surpris, la main ouverte. Puis il penche la tête. Il cherche sous la feuille. Là. La fraise rouge est là, tiède. Il la cueille, sans se presser. Elle est à moi. Elle pèse dans sa paume. Elle est tiède, un peu molle. Elle chauffe ma main. Elle est tiède, Chouchou ? Oui, maman. Un sourire arrive sur son visage. Ses joues deviennent chaudes. Sa poitrine se remplit, chaude. Dans sa poitrine, c'est plein. Ses épaules se lèvent un peu. Papa s'accroupit à la même hauteur. Tu vois la fraise, Chouchou ? Oui, papa. Tes joues sont chaudes, Chouchou ? Un peu, maman. L'éclat de treille tremble, sous le fil.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un petit panier attend près du gravier. Dedans, un torchon à carreaux. Les fraisiers cachent des fruits. Les feuilles sont vertes. Un peu piquantes. La terre est chaude. L'arrosoir de papa goutte encore. Je pose le panier, Chouchou. On marche tout doux, entre les plants. Ça sent le sucre, papa. Oui. Les fraises sont mûres. Le soleil est doux, ce matin. Regarde sous les feuilles. En ce moment, Chouchou marche. Il est près des fraisiers. Papa est là, près de lui. Chouchou voit une fraise rouge. Une fraise ! Elle brille. Tu la cueilles tout doucement ? Une seule, pour commencer. Chouchou cueille la fraise. Tout doucement. La fraise sent le sucre. Elle est tiède dans sa main. Chouchou sent ses joues chaudes. Son ventre est léger. Un sourire arrive. Je suis content. C'est de la joie. Tu es content. Tes joues sont chaudes. Oui. De la joie. On peut partager. Chouchou tend la fraise. Un bout pour papa. Et un tout petit bout pour toi. Papa prend un tout petit bout. Chouchou prend un tout petit bout. Merci, Chouchou. Tu as partagé. Je suis content. La joie est là, dans le jardin. Ils sourient ensemble. La terre reste chaude. L'arrosoir goutte encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La treille du fond fait de l'ombre. Elle fait de l'ombre, papa. Tu la vois, la treille ? Oui, papa. Un fil de fer vibre sous le pouce. Ting, près du bois. Tu entends le fil, Chouchou ? Oui, maman. Maman s'assoit près du fil. La terre chauffe les genoux. Elle est chaude. Les genoux sont bien ? Oui, maman. Papa soulève une feuille de vigne. Le bois sent le soleil. Tu sens le bois chaud ? Oui, papa. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de treille&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le bois ? Oui, un petit point. Le soleil le touche. Un rayon glisse sur le bord. La treille chauffe le jardin. Elle est chaude. Tu poses la main, Chouchou ? Oui. Une fraise rouge attend sous la feuille. Une fraise ! Elle est rouge, Chouchou ? Oui, maman. Elle sent un peu le sucre. Ça sent le sucre, papa. Tu la veux, la fraise ? Oui, maintenant ! En ce moment, Chouchou tend la main. Je la prends, tout de suite ! Tout de suite ? Oui, papa. Chouchou attrape trop vite. Sa main prend la feuille. Oh. La fraise reste cachée. Les doigts tiennent du vert. La feuille, pas la fraise ? Pas la fraise. Chouchou reste surpris, la main ouverte. Puis il penche la tête. Il cherche sous la feuille. Là. La fraise rouge est là, tiède. Il la cueille, sans se presser. Elle est à moi. Elle pèse dans sa paume. Elle est tiède, un peu molle. Elle chauffe ma main. Elle est tiède, Chouchou ? Oui, maman. Un sourire arrive sur son visage. Ses joues deviennent chaudes. Sa poitrine se remplit, chaude. Dans sa poitrine, c'est plein. Ses épaules se lèvent un peu. Papa s'accroupit à la même hauteur. Tu vois la fraise, Chouchou ? Oui, papa. Tes joues sont chaudes, Chouchou ? Un peu, maman. L'éclat de treille tremble, sous le fil.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Tom marche dans le jardin. Papa est là, près des fraisiers. Le soleil est doux. Tom voit une fraise rouge. Il la cueille tout doucement. La fraise sent le sucre. Tom sent ses joues chaudes. Son ventre est léger. Un sourire arrive. Tom dit : je suis &lt;emphasis&gt;content&lt;/emphasis&gt;. Papa dit : c'est de la joie. Tom tend la fraise. Il dit : on peut partager. Papa prend un tout petit bout. Tom prend un tout petit bout. Ils sourient ensemble. Tom dit encore : je suis content. La joie est là, dans le jardin.&lt;/slow&gt; [pause]</t>
+          <t>La treille du fond fait de l'ombre. Elle fait de l'ombre, papa. Tu la vois, la treille ? Oui, papa. Un fil de fer vibre sous le pouce. Ting, près du bois. Tu entends le fil, Chouchou ? Oui, maman. Maman s'assoit près du fil. La terre chauffe les genoux. Elle est chaude. Les genoux sont bien ? Oui, maman. Papa soulève une feuille de vigne. Le bois sent le soleil. Tu sens le bois chaud ? Oui, papa. Sur le bois, un &lt;emphasis&gt;éclat de treille&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le bois ? Oui, un petit point. Le soleil le touche. Un rayon glisse sur le bord. La treille chauffe le jardin. Elle est chaude. Tu poses la main, Chouchou ? Oui. Une fraise rouge attend sous la feuille. Une fraise ! Elle est rouge, Chouchou ? Oui, maman. Elle sent un peu le sucre. Ça sent le sucre, papa. Tu la veux, la fraise ? Oui, maintenant ! En ce moment, Chouchou tend la main. Je la prends, tout de suite ! Tout de suite ? Oui, papa. Chouchou attrape trop vite. Sa main prend la feuille. Oh. La fraise reste cachée. Les doigts tiennent du vert. La feuille, pas la fraise ? Pas la fraise. Chouchou reste surpris, la main ouverte. Puis il penche la tête. Il cherche sous la feuille. Là. La fraise rouge est là, tiède. Il la cueille, sans se presser. Elle est à moi. Elle pèse dans sa paume. Elle est tiède, un peu molle. Elle chauffe ma main. Elle est tiède, Chouchou ? Oui, maman. Un sourire arrive sur son visage. Ses joues deviennent chaudes. Sa poitrine se remplit, chaude. Dans sa poitrine, c'est plein. Ses épaules se lèvent un peu. Papa s'accroupit à la même hauteur. Tu vois la fraise, Chouchou ? Oui, papa. Tes joues sont chaudes, Chouchou ? Un peu, maman. L'éclat de treille tremble, sous le fil. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,18 +1241,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>content</t>
+          <t>éclat de treille</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,54 +1319,84 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis joie; intensite=2; destinataire=enfant; sous_texte=il_veut_la_fraise_maintenant; tempo=posé puis resserré; sourire=aucun puis qui_arrive; respiration=ample puis pleine</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un petit panier attend près du gravier.
-narrateur|Dedans, un torchon à carreaux.
-narrateur|Les fraisiers cachent des fruits.
-narrateur|Les feuilles sont vertes.
-narrateur|Un peu piquantes.
-narrateur|La terre est chaude.
-narrateur|L'arrosoir de papa goutte encore.
-maman|Je pose le panier, Chouchou.
-papa|On marche tout doux, entre les plants.
+          <t>narrateur|La treille du fond fait de l'ombre.
+enfant-m|Elle fait de l'ombre, papa.
+papa|Tu la vois, la treille ?
+enfant-m|Oui, papa.
+narrateur|Un fil de fer vibre sous le pouce.
+narrateur|Ting, près du bois.
+maman|Tu entends le fil, Chouchou ?
+enfant-m|Oui, maman.
+narrateur|Maman s'assoit près du fil.
+narrateur|La terre chauffe les genoux.
+enfant-m|Elle est chaude.
+maman|Les genoux sont bien ?
+enfant-m|Oui, maman.
+narrateur|Papa soulève une feuille de vigne.
+narrateur|Le bois sent le soleil.
+papa|Tu sens le bois chaud ?
+enfant-m|Oui, papa.
+narrateur|Sur le bois, un éclat de treille luit.
+enfant-m|Il brille, maman.
+maman|Tu le vois, sur le bois ?
+enfant-m|Oui, un petit point.
+papa|Le soleil le touche.
+narrateur|Un rayon glisse sur le bord.
+narrateur|La treille chauffe le jardin.
+enfant-m|Elle est chaude.
+maman|Tu poses la main, Chouchou ?
+enfant-m|Oui.
+narrateur|Une fraise rouge attend sous la feuille.
+enfant-m|Une fraise !
+maman|Elle est rouge, Chouchou ?
+enfant-m|Oui, maman.
+narrateur|Elle sent un peu le sucre.
 enfant-m|Ça sent le sucre, papa.
-papa|Oui. Les fraises sont mûres.
-maman|Le soleil est doux, ce matin.
-papa|Regarde sous les feuilles.
-narrateur|En ce moment, Chouchou marche.
-narrateur|Il est près des fraisiers.
-narrateur|Papa est là, près de lui.
-narrateur|Chouchou voit une fraise rouge.
-enfant-m|Une fraise ! Elle brille.
-papa|Tu la cueilles tout doucement ?
-maman|Une seule, pour commencer.
-narrateur|Chouchou cueille la fraise.
-narrateur|Tout doucement.
-narrateur|La fraise sent le sucre.
-narrateur|Elle est tiède dans sa main.
-narrateur|Chouchou sent ses joues chaudes.
-narrateur|Son ventre est léger.
-narrateur|Un sourire arrive.
-enfant-m|Je suis content.
-papa|C'est de la joie.
-maman|Tu es content. Tes joues sont chaudes.
-enfant-m|Oui. De la joie.
-papa|On peut partager.
-narrateur|Chouchou tend la fraise.
-enfant-m|Un bout pour papa.
-maman|Et un tout petit bout pour toi.
-narrateur|Papa prend un tout petit bout.
-narrateur|Chouchou prend un tout petit bout.
-papa|Merci, Chouchou. Tu as partagé.
-enfant-m|Je suis content.
-maman|La joie est là, dans le jardin.
-narrateur|Ils sourient ensemble.
-narrateur|La terre reste chaude.
-narrateur|L'arrosoir goutte encore.</t>
+papa|Tu la veux, la fraise ?
+enfant-m|Oui, maintenant !
+narrateur|En ce moment, Chouchou tend la main.
+enfant-m|Je la prends, tout de suite !
+papa|Tout de suite ?
+enfant-m|Oui, papa.
+narrateur|Chouchou attrape trop vite.
+narrateur|Sa main prend la feuille.
+enfant-m|Oh.
+narrateur|La fraise reste cachée.
+narrateur|Les doigts tiennent du vert.
+maman|La feuille, pas la fraise ?
+enfant-m|Pas la fraise.
+narrateur|Chouchou reste surpris, la main ouverte.
+narrateur|Puis il penche la tête.
+narrateur|Il cherche sous la feuille.
+enfant-m|Là.
+narrateur|La fraise rouge est là, tiède.
+narrateur|Il la cueille, sans se presser.
+enfant-m|Elle est à moi.
+narrateur|Elle pèse dans sa paume.
+narrateur|Elle est tiède, un peu molle.
+enfant-m|Elle chauffe ma main.
+maman|Elle est tiède, Chouchou ?
+enfant-m|Oui, maman.
+narrateur|Un sourire arrive sur son visage.
+narrateur|Ses joues deviennent chaudes.
+narrateur|Sa poitrine se remplit, chaude.
+narrateur|Dans sa poitrine, c'est plein.
+narrateur|Ses épaules se lèvent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois la fraise, Chouchou ?
+enfant-m|Oui, papa.
+maman|Tes joues sont chaudes, Chouchou ?
+enfant-m|Un peu, maman.
+narrateur|L'éclat de treille tremble, sous le fil.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1403,12 +1433,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Chouchou sourit. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;&lt;emphasis level="moderate"&gt;Chouchou&lt;/emphasis&gt; sourit. Que dit-il ?&lt;/prosody&gt;&lt;break time="780ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Tom sourit. Que dit-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;&lt;emphasis&gt;Chouchou&lt;/emphasis&gt; sourit. Que dit-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1433,7 +1463,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Tom sent de la joie. Que dit-il ?</t>
+          <t>Chouchou sent de la joie. Que dit-il ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1471,7 +1501,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1482,7 +1512,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1497,34 +1527,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Chouchou</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>780</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.3</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1539,7 +1573,7 @@
         <v>0.8</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1549,7 +1583,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=chouchou_sourit_que_dit_il; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1582,17 +1616,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou a nommé sa joie. Il a partagé avec papa. Je suis content. Oui. C'est de la joie. Tu as tendu la fraise. Bravo. Chouchou essuie ses doigts. Le jus est un peu rouge. Ça sent encore le sucre. On met le panier près des plants ? Oui. Encore une fraise, plus tard. On peut inviter papa à goûter encore. Viens, papa. Un tout petit bout. Merci. On partage. Tu as dit : je suis content. C'est bien. C'est de la joie, maman. La joie se partage. Tu as invité.</t>
+          <t>Chouchou serre la fraise, trop fort. Je la mange, maintenant ! Le jus glisse entre ses doigts. Les mots se bousculent dans sa bouche. Trop vite. Il avance la fraise vers sa bouche. Puis il s'arrête. Il referme la bouche. Personne ne parle. Il observe la fraise, un instant. Il écoute le jardin. Je suis content. Sa voix est petite, près de la fraise. Tu restes un peu, Chouchou ? Oui, papa. Chouchou tend la fraise vers papa. Un bout pour toi. Papa prend un petit bout. Merci, Chouchou. Papa reste à la même hauteur. Le jus est rouge, sous les doigts. Il est sucré. Chouchou garde un bout, dans la paume. Tu le vois, le bout ? Oui, papa. Il est tiède, Chouchou ? Oui, maman. Le sourire reste près de la fraise. Je suis content. Les joues sont chaudes ? Oui, papa. Tes mains sont rouges ? Un peu, maman. Le ventre de Chouchou se desserre. Les épaules restent hautes. On reste près de la treille ? Oui. Le rayon touche le bois ? Oui, maman. La fraise attend dans sa main. Je la tiens. Tu la tiens, Chouchou ? Oui, papa.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou a nommé sa joie. Il a partagé avec papa. Je suis content. Oui. C'est de la joie. Tu as tendu la fraise. Bravo. Chouchou essuie ses doigts. Le jus est un peu rouge. Ça sent encore le sucre. On met le panier près des plants ? Oui. Encore une fraise, plus tard. On peut inviter papa à goûter encore. Viens, papa. Un tout petit bout. Merci. On partage. Tu as dit : je suis content. C'est bien. C'est de la joie, maman. La joie se partage. Tu as invité.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Chouchou serre la fraise, trop fort. Je la mange, maintenant ! Le jus glisse entre ses doigts. Les mots se bousculent dans sa bouche. Trop vite. Il avance la fraise vers sa bouche. Puis il s'arrête. Il referme la bouche. Personne ne parle. Il observe la fraise, un instant. Il écoute le jardin. Je suis &lt;emphasis level="moderate"&gt;content&lt;/emphasis&gt;. Sa voix est petite, près de la fraise. Tu restes un peu, Chouchou ? Oui, papa. Chouchou tend la fraise vers papa. Un bout pour toi. Papa prend un petit bout. Merci, Chouchou. Papa reste à la même hauteur. Le jus est rouge, sous les doigts. Il est sucré. Chouchou garde un bout, dans la paume. Tu le vois, le bout ? Oui, papa. Il est tiède, Chouchou ? Oui, maman. Le sourire reste près de la fraise. Je suis content. Les joues sont chaudes ? Oui, papa. Tes mains sont rouges ? Un peu, maman. Le ventre de Chouchou se desserre. Les épaules restent hautes. On reste près de la treille ? Oui. Le rayon touche le bois ? Oui, maman. La fraise attend dans sa main. Je la tiens. Tu la tiens, Chouchou ? Oui, papa.&lt;/prosody&gt;&lt;break time="620ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Tom a nommé sa joie. Il a partagé avec papa. Être &lt;emphasis&gt;content&lt;/emphasis&gt;, c'est bien.&lt;/slow&gt; [pause]</t>
+          <t>Chouchou serre la fraise, trop fort. Je la mange, maintenant ! Le jus glisse entre ses doigts. Les mots se bousculent dans sa bouche. Trop vite. Il avance la fraise vers sa bouche. Puis il s'arrête. Il referme la bouche. Personne ne parle. Il observe la fraise, un instant. Il écoute le jardin. Je suis &lt;emphasis&gt;content&lt;/emphasis&gt;. Sa voix est petite, près de la fraise. Tu restes un peu, Chouchou ? Oui, papa. Chouchou tend la fraise vers papa. Un bout pour toi. Papa prend un petit bout. Merci, Chouchou. Papa reste à la même hauteur. Le jus est rouge, sous les doigts. Il est sucré. Chouchou garde un bout, dans la paume. Tu le vois, le bout ? Oui, papa. Il est tiède, Chouchou ? Oui, maman. Le sourire reste près de la fraise. Je suis content. Les joues sont chaudes ? Oui, papa. Tes mains sont rouges ? Un peu, maman. Le ventre de Chouchou se desserre. Les épaules restent hautes. On reste près de la treille ? Oui. Le rayon touche le bois ? Oui, maman. La fraise attend dans sa main. Je la tiens. Tu la tiens, Chouchou ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1639,18 +1673,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.24</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1680,23 +1714,23 @@
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>620</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>310</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.33</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1705,10 +1739,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1717,31 +1751,58 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=joie puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_dit_je_suis_content_il_tend_un_bout; tempo=posé; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou a nommé sa joie.
-narrateur|Il a partagé avec papa.
+          <t>narrateur|Chouchou serre la fraise, trop fort.
+enfant-m|Je la mange, maintenant !
+narrateur|Le jus glisse entre ses doigts.
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-m|Trop vite.
+narrateur|Il avance la fraise vers sa bouche.
+narrateur|Puis il s'arrête.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe la fraise, un instant.
+narrateur|Il écoute le jardin.
 enfant-m|Je suis content.
-papa|Oui. C'est de la joie.
-maman|Tu as tendu la fraise. Bravo.
-narrateur|Chouchou essuie ses doigts.
-narrateur|Le jus est un peu rouge.
-narrateur|Ça sent encore le sucre.
-papa|On met le panier près des plants ?
-enfant-m|Oui. Encore une fraise, plus tard.
-maman|On peut inviter papa à goûter encore.
-enfant-m|Viens, papa. Un tout petit bout.
-papa|Merci. On partage.
-maman|Tu as dit : je suis content. C'est bien.
-enfant-m|C'est de la joie, maman.
-papa|La joie se partage. Tu as invité.</t>
+narrateur|Sa voix est petite, près de la fraise.
+papa|Tu restes un peu, Chouchou ?
+enfant-m|Oui, papa.
+narrateur|Chouchou tend la fraise vers papa.
+enfant-m|Un bout pour toi.
+narrateur|Papa prend un petit bout.
+papa|Merci, Chouchou.
+narrateur|Papa reste à la même hauteur.
+maman|Le jus est rouge, sous les doigts.
+enfant-m|Il est sucré.
+narrateur|Chouchou garde un bout, dans la paume.
+papa|Tu le vois, le bout ?
+enfant-m|Oui, papa.
+maman|Il est tiède, Chouchou ?
+enfant-m|Oui, maman.
+narrateur|Le sourire reste près de la fraise.
+enfant-m|Je suis content.
+papa|Les joues sont chaudes ?
+enfant-m|Oui, papa.
+maman|Tes mains sont rouges ?
+enfant-m|Un peu, maman.
+narrateur|Le ventre de Chouchou se desserre.
+narrateur|Les épaules restent hautes.
+papa|On reste près de la treille ?
+enfant-m|Oui.
+maman|Le rayon touche le bois ?
+enfant-m|Oui, maman.
+narrateur|La fraise attend dans sa main.
+enfant-m|Je la tiens.
+papa|Tu la tiens, Chouchou ?
+enfant-m|Oui, papa.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1773,17 +1834,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Chouchou essuie ses mains. Le jardin est calme. Tu me prends la main ? Oui, papa. Le panier est là. Merci, Chouchou. Je suis content. C'est de la joie. Tu as partagé. On rentre avec le panier ? Oui. La fraise était sucrée. Ils marchent vers la maison. Les graviers font un petit bruit. Tu as invité papa. Bravo. On pose le panier près de la porte ? Oui. Je suis encore content. L'arrosoir reste près des plants.</t>
+          <t>Maman se baisse près de la treille. La fraise brille, trop chaude. Un bout pour toi, maman ! Chouchou tend la fraise, trop vite. Elle glisse de sa main. Elle tombe ! La fraise penche vers la terre. Chouchou avance les mains, trop vite. Puis il s'arrête net. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la fraise, un instant. Il écoute le jardin, près du fil. Sur le bois, un éclat de treille luit. Là, sur le bois. Il attend, les deux mains ouvertes. On tient la fraise ? Oui, papa. La fraise sent le sucre chaud. Elle est là, un peu penchée. Chouchou la reprend, sans se presser. Il la casse en deux. Pour toi. Le jus est tiède, Chouchou ? Un peu. Il tend un bout vers maman. Pour moi ? Oui, maman. Le bout tient, Chouchou ? Oui, papa. Un rayon passe sur le bois. Il allume le fil. Tu vois le point, Chouchou ? Oui, papa. Maman prend le bout, près des lèvres. Il est sucré. La treille est calme ? Oui, papa. Tes genoux sont au chaud ? Un peu, maman. Le bois reste proche, près d'eux. Il sent le soleil. On reste ici, Chouchou ? Oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Chouchou essuie ses mains. Le jardin est calme. Tu me prends la main ? Oui, papa. Le panier est là. Merci, Chouchou. Je suis content. C'est de la joie. Tu as partagé. On rentre avec le panier ? Oui. La fraise était sucrée. Ils marchent vers la maison. Les graviers font un petit bruit. Tu as invité papa. Bravo. On pose le panier près de la porte ? Oui. Je suis encore content. L'arrosoir reste près des plants.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman se baisse près de la treille. La fraise brille, trop chaude. Un bout pour toi, maman ! Chouchou tend la fraise, trop vite. Elle glisse de sa main. Elle tombe ! La fraise penche vers la terre. Chouchou avance les mains, trop vite. Puis il s'arrête net. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la fraise, un instant. Il écoute le jardin, près du fil. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de treille&lt;/emphasis&gt; luit. Là, sur le bois. Il attend, les deux mains ouvertes. On tient la fraise ? Oui, papa. La fraise sent le sucre chaud. Elle est là, un peu penchée. Chouchou la reprend, sans se presser. Il la casse en deux. Pour toi. Le jus est tiède, Chouchou ? Un peu. Il tend un bout vers maman. Pour moi ? Oui, maman. Le bout tient, Chouchou ? Oui, papa. Un rayon passe sur le bois. Il allume le fil. Tu vois le point, Chouchou ? Oui, papa. Maman prend le bout, près des lèvres. Il est sucré. La treille est calme ? Oui, papa. Tes genoux sont au chaud ? Un peu, maman. Le bois reste proche, près d'eux. Il sent le soleil. On reste ici, Chouchou ? Oui.&lt;/prosody&gt;&lt;break time="480ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Tom essuie ses &lt;emphasis&gt;main&lt;/emphasis&gt;s. Le jardin est calme. Papa lui prend la main.&lt;/slow&gt; [pause]</t>
+          <t>Maman se baisse près de la treille. La fraise brille, trop chaude. Un bout pour toi, maman ! Chouchou tend la fraise, trop vite. Elle glisse de sa main. Elle tombe ! La fraise penche vers la terre. Chouchou avance les mains, trop vite. Puis il s'arrête net. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la fraise, un instant. Il écoute le jardin, près du fil. Sur le bois, un &lt;emphasis&gt;éclat de treille&lt;/emphasis&gt; luit. Là, sur le bois. Il attend, les deux mains ouvertes. On tient la fraise ? Oui, papa. La fraise sent le sucre chaud. Elle est là, un peu penchée. Chouchou la reprend, sans se presser. Il la casse en deux. Pour toi. Le jus est tiède, Chouchou ? Un peu. Il tend un bout vers maman. Pour moi ? Oui, maman. Le bout tient, Chouchou ? Oui, papa. Un rayon passe sur le bois. Il allume le fil. Tu vois le point, Chouchou ? Oui, papa. Maman prend le bout, près des lèvres. Il est sucré. La treille est calme ? Oui, papa. Tes genoux sont au chaud ? Un peu, maman. Le bois reste proche, près d'eux. Il sent le soleil. On reste ici, Chouchou ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1830,18 +1891,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1864,30 +1925,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de treille</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1896,10 +1957,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1908,31 +1969,65 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=la_fraise_glisse_trop_chaude_il_s_arrete; tempo=un peu vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou essuie ses mains.
-narrateur|Le jardin est calme.
-papa|Tu me prends la main ?
+          <t>narrateur|Maman se baisse près de la treille.
+narrateur|La fraise brille, trop chaude.
+enfant-m|Un bout pour toi, maman !
+narrateur|Chouchou tend la fraise, trop vite.
+narrateur|Elle glisse de sa main.
+enfant-m|Elle tombe !
+narrateur|La fraise penche vers la terre.
+narrateur|Chouchou avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Chouchou refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe la fraise, un instant.
+narrateur|Il écoute le jardin, près du fil.
+narrateur|Sur le bois, un éclat de treille luit.
+enfant-m|Là, sur le bois.
+narrateur|Il attend, les deux mains ouvertes.
+papa|On tient la fraise ?
 enfant-m|Oui, papa.
-maman|Le panier est là. Merci, Chouchou.
-enfant-m|Je suis content.
-papa|C'est de la joie. Tu as partagé.
-maman|On rentre avec le panier ?
-enfant-m|Oui. La fraise était sucrée.
-narrateur|Ils marchent vers la maison.
-narrateur|Les graviers font un petit bruit.
-maman|Tu as invité papa. Bravo.
-papa|On pose le panier près de la porte ?
-enfant-m|Oui. Je suis encore content.
-narrateur|L'arrosoir reste près des plants.</t>
+narrateur|La fraise sent le sucre chaud.
+narrateur|Elle est là, un peu penchée.
+narrateur|Chouchou la reprend, sans se presser.
+narrateur|Il la casse en deux.
+enfant-m|Pour toi.
+maman|Le jus est tiède, Chouchou ?
+enfant-m|Un peu.
+narrateur|Il tend un bout vers maman.
+maman|Pour moi ?
+enfant-m|Oui, maman.
+papa|Le bout tient, Chouchou ?
+enfant-m|Oui, papa.
+maman|Un rayon passe sur le bois.
+enfant-m|Il allume le fil.
+papa|Tu vois le point, Chouchou ?
+enfant-m|Oui, papa.
+narrateur|Maman prend le bout, près des lèvres.
+enfant-m|Il est sucré.
+papa|La treille est calme ?
+enfant-m|Oui, papa.
+maman|Tes genoux sont au chaud ?
+enfant-m|Un peu, maman.
+narrateur|Le bois reste proche, près d'eux.
+enfant-m|Il sent le soleil.
+papa|On reste ici, Chouchou ?
+enfant-m|Oui.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>jardin</t>
+          <t>jardin,fraise</t>
         </is>
       </c>
     </row>
@@ -1959,17 +2054,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'étais content. C'était de la joie. Tu as partagé. Bravo. La fraise était rouge. Le jardin était calme.</t>
+          <t>Ils restent près de la treille. Maman essuie un peu de jus. La fraise a glissé, papa. Tu l'as vue, toi ? Oui, près de la terre. On est bien, ici. Chouchou tapote le bois du doigt. Il a une trace de jus. Tu la vois, la trace ? Oui, maman. La fraise est restée, Chouchou. Oui, avec un bout. Ça sent le sucre, un peu tiède. Et le bois, maman. Oui, dans l'air. Le jardin est calme, Chouchou ? Oui, papa. La fraise reste dans la paume. Un éclat de treille tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'étais content. C'était de la joie. Tu as partagé. Bravo. La fraise était rouge. Le jardin était calme.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la treille. Maman essuie un peu de jus. La fraise a glissé, papa. Tu l'as vue, toi ? Oui, près de la terre. On est bien, ici. Chouchou tapote le bois du doigt. Il a une trace de jus. Tu la vois, la trace ? Oui, maman. La fraise est restée, Chouchou. Oui, avec un bout. Ça sent le sucre, un peu tiède. Et le bois, maman. Oui, dans l'air. Le jardin est calme, Chouchou ? Oui, papa. La fraise reste dans la paume. Un &lt;emphasis level="moderate"&gt;éclat de treille&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="980ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la treille. Maman essuie un peu de jus. La fraise a glissé, papa. Tu l'as vue, toi ? Oui, près de la terre. On est bien, ici. Chouchou tapote le bois du doigt. Il a une trace de jus. Tu la vois, la trace ? Oui, maman. La fraise est restée, Chouchou. Oui, avec un bout. Ça sent le sucre, un peu tiède. Et le bois, maman. Oui, dans l'air. Le jardin est calme, Chouchou ? Oui, papa. La fraise reste dans la paume. Un &lt;emphasis&gt;éclat de treille&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2016,7 +2111,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2024,7 +2119,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.36</v>
@@ -2036,12 +2131,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2050,14 +2145,18 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de treille</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>980</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>380</v>
@@ -2069,11 +2168,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.29</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2082,26 +2181,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'étais content. C'était de la joie.
-papa|Tu as partagé. Bravo.
-maman|La fraise était rouge. Le jardin était calme.</t>
+          <t>narrateur|Ils restent près de la treille.
+narrateur|Maman essuie un peu de jus.
+enfant-m|La fraise a glissé, papa.
+papa|Tu l'as vue, toi ?
+enfant-m|Oui, près de la terre.
+maman|On est bien, ici.
+narrateur|Chouchou tapote le bois du doigt.
+enfant-m|Il a une trace de jus.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|La fraise est restée, Chouchou.
+enfant-m|Oui, avec un bout.
+narrateur|Ça sent le sucre, un peu tiède.
+enfant-m|Et le bois, maman.
+maman|Oui, dans l'air.
+papa|Le jardin est calme, Chouchou ?
+enfant-m|Oui, papa.
+narrateur|La fraise reste dans la paume.
+narrateur|Un éclat de treille tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2186,6 +2305,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>